<commit_message>
checkpoint: R16.1 consolidation 2026-08-16T23:16Z
</commit_message>
<xml_diff>
--- a/outputs/TRUE-CLOUD-MIGRATION/01_REQUIREMENTS_REGISTER.xlsx
+++ b/outputs/TRUE-CLOUD-MIGRATION/01_REQUIREMENTS_REGISTER.xlsx
@@ -9,7 +9,10 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Requirements'!$A$4:$I$15</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Requirements'!$1:$4</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +28,31 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00374151"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,12 +67,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -411,576 +449,617 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>True Cloud Migration — Requirement Register</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Current working register · Generated 2026-08-16T06:30:42+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Track</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Clarification</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Assumption</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Domains</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>REQ-T1-001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>AWS Legacy Zone HLD/LLD</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>ARCHITECTURE</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>DESIGN_DOCUMENT</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>SOW</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>account structure,network segmentation,security,routing,logging,monitoring,governance</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>REQ-T1-002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>AWS Landing Zone / Legacy Zone As-Built</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>ARCHITECTURE</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>AS_BUILT</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>SOW</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>landing zone,legacy zone,thailand region</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>REQ-T1-003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Core Infrastructure Services Design / As-Built</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>IDENTITY</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>DESIGN_AND_AS_BUILT</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>SOW</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>active directory,dns,firewall,jump host,cyberark</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>REQ-T1-004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Jump Host Migration</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>MIGRATION</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>MIGRATED_SERVERS</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>SOW</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>jump host</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>REQ-T1-005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>CyberArk Migration</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>MIGRATION</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>MIGRATED_SERVERS</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>SOW</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>cyberark</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>REQ-T1-006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>T1</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Hybrid / Multi-cloud Connectivity Assessment</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>CONNECTIVITY</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>ASSESSMENT</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>SOW</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>on-premises,direct connect,azure,gcp,hybrid,multi-cloud</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>REQ-T2-001</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Migration Factory Design</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>MIGRATION</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>DESIGN_DOCUMENT</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>SOW</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>staging subnet,routing,vpc endpoint</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>REQ-T2-002</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Migration Network Foundation As-Built</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>NETWORK</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>AS_BUILT</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>SOW</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>subnets,route tables,direct connect,privatelink,security groups</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>REQ-T2-003</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>AWS MGN Agent Enablement / Configuration</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>MIGRATION</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>CONFIG_SUMMARY</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>SOW</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>dns resolution,endpoint usage,agent installation</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>REQ-T2-004</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Pilot Migration Test / Verification</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>TEST / VERIFICATION</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>TEST_REPORT</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>SOW</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>private-path migration,health status</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>REQ-T2-005</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Migration Runbook / Operational Handover</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>OPERATIONS</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>RUNBOOK</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>SOW</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>NONE</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>migration waves,migration factory execution</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:I15"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G5:G15">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>G5="OPEN"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H5:H15">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>H5="OPEN"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>